<commit_message>
Add original order placement dates to recovery report
Update Excel report to include the original creation date for each cancelled order associated with recovery deductions.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 7cdd434c-ed09-4143-9d63-3c20e2d8d6b0
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: aee02868-457a-438b-9db9-ba0d211632e2
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/348b80b5-3718-405c-9777-744d35985801/7cdd434c-ed09-4143-9d63-3c20e2d8d6b0/hRxk6j6
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/over_refund_recovery_20Jul2026.xlsx
+++ b/over_refund_recovery_20Jul2026.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Recovery Deductions Jul 20" sheetId="1" r:id="rId1"/>
+    <sheet name="Order Breakdown" sheetId="1" r:id="rId1"/>
+    <sheet name="Agent Summary" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -397,28 +398,627 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F29"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="25.83203125" customWidth="1"/>
-    <col min="5" max="5" width="25.83203125" customWidth="1"/>
-    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Agent Name</v>
+        <v>Agent</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Order ID</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Order Placed Date</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Amount Refunded (GHS)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Correct Refund (GHS)</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Over-Refund Recovered (GHS)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Dela Kwesi</v>
+      </c>
+      <c r="B2" t="str">
+        <v>ORD-082506</v>
+      </c>
+      <c r="C2" t="str">
+        <v>15-Jul-2026</v>
+      </c>
+      <c r="D2">
+        <v>12</v>
+      </c>
+      <c r="E2">
+        <v>4</v>
+      </c>
+      <c r="F2">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Emmanuel Simpson</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ORD-084475</v>
+      </c>
+      <c r="C3" t="str">
+        <v>18-Jul-2026</v>
+      </c>
+      <c r="D3">
+        <v>80</v>
+      </c>
+      <c r="E3">
+        <v>40</v>
+      </c>
+      <c r="F3">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Flashdealsgh</v>
+      </c>
+      <c r="B4" t="str">
+        <v>ORD-082068</v>
+      </c>
+      <c r="C4" t="str">
+        <v>14-Jul-2026</v>
+      </c>
+      <c r="D4">
+        <v>16</v>
+      </c>
+      <c r="E4">
+        <v>4</v>
+      </c>
+      <c r="F4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Flashdealsgh</v>
+      </c>
+      <c r="B5" t="str">
+        <v>ORD-082673</v>
+      </c>
+      <c r="C5" t="str">
+        <v>15-Jul-2026</v>
+      </c>
+      <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Flashdealsgh</v>
+      </c>
+      <c r="B6" t="str">
+        <v>ORD-082739</v>
+      </c>
+      <c r="C6" t="str">
+        <v>15-Jul-2026</v>
+      </c>
+      <c r="D6">
+        <v>47.5</v>
+      </c>
+      <c r="E6">
+        <v>39.5</v>
+      </c>
+      <c r="F6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Flashdealsgh</v>
+      </c>
+      <c r="B7" t="str">
+        <v>ORD-082838</v>
+      </c>
+      <c r="C7" t="str">
+        <v>16-Jul-2026</v>
+      </c>
+      <c r="D7">
+        <v>20</v>
+      </c>
+      <c r="E7">
+        <v>8</v>
+      </c>
+      <c r="F7">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Flashdealsgh</v>
+      </c>
+      <c r="B8" t="str">
+        <v>ORD-083155</v>
+      </c>
+      <c r="C8" t="str">
+        <v>16-Jul-2026</v>
+      </c>
+      <c r="D8">
+        <v>8</v>
+      </c>
+      <c r="E8">
+        <v>4</v>
+      </c>
+      <c r="F8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Flashdealsgh</v>
+      </c>
+      <c r="B9" t="str">
+        <v>ORD-083419</v>
+      </c>
+      <c r="C9" t="str">
+        <v>16-Jul-2026</v>
+      </c>
+      <c r="D9">
+        <v>24</v>
+      </c>
+      <c r="E9">
+        <v>16</v>
+      </c>
+      <c r="F9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Flashdealsgh</v>
+      </c>
+      <c r="B10" t="str">
+        <v>ORD-083485</v>
+      </c>
+      <c r="C10" t="str">
+        <v>17-Jul-2026</v>
+      </c>
+      <c r="D10">
+        <v>44</v>
+      </c>
+      <c r="E10">
+        <v>4</v>
+      </c>
+      <c r="F10">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Flashdealsgh</v>
+      </c>
+      <c r="B11" t="str">
+        <v>ORD-083539</v>
+      </c>
+      <c r="C11" t="str">
+        <v>17-Jul-2026</v>
+      </c>
+      <c r="D11">
+        <v>73</v>
+      </c>
+      <c r="E11">
+        <v>4</v>
+      </c>
+      <c r="F11">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Flashdealsgh</v>
+      </c>
+      <c r="B12" t="str">
+        <v>ORD-084002</v>
+      </c>
+      <c r="C12" t="str">
+        <v>17-Jul-2026</v>
+      </c>
+      <c r="D12">
+        <v>191</v>
+      </c>
+      <c r="E12">
+        <v>20</v>
+      </c>
+      <c r="F12">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Flashdealsgh</v>
+      </c>
+      <c r="B13" t="str">
+        <v>ORD-084042</v>
+      </c>
+      <c r="C13" t="str">
+        <v>17-Jul-2026</v>
+      </c>
+      <c r="D13">
+        <v>36</v>
+      </c>
+      <c r="E13">
+        <v>4</v>
+      </c>
+      <c r="F13">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Flashdealsgh</v>
+      </c>
+      <c r="B14" t="str">
+        <v>ORD-084241</v>
+      </c>
+      <c r="C14" t="str">
+        <v>18-Jul-2026</v>
+      </c>
+      <c r="D14">
+        <v>279.5</v>
+      </c>
+      <c r="E14">
+        <v>4.1</v>
+      </c>
+      <c r="F14">
+        <v>275.4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Flashdealsgh</v>
+      </c>
+      <c r="B15" t="str">
+        <v>ORD-084592</v>
+      </c>
+      <c r="C15" t="str">
+        <v>18-Jul-2026</v>
+      </c>
+      <c r="D15">
+        <v>16.4</v>
+      </c>
+      <c r="E15">
+        <v>4.1</v>
+      </c>
+      <c r="F15">
+        <v>12.3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Kenneth</v>
+      </c>
+      <c r="B16" t="str">
+        <v>ORD-083558</v>
+      </c>
+      <c r="C16" t="str">
+        <v>17-Jul-2026</v>
+      </c>
+      <c r="D16">
+        <v>116</v>
+      </c>
+      <c r="E16">
+        <v>4</v>
+      </c>
+      <c r="F16">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Kenneth</v>
+      </c>
+      <c r="B17" t="str">
+        <v>ORD-083636</v>
+      </c>
+      <c r="C17" t="str">
+        <v>17-Jul-2026</v>
+      </c>
+      <c r="D17">
+        <v>24</v>
+      </c>
+      <c r="E17">
+        <v>4</v>
+      </c>
+      <c r="F17">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Kenneth</v>
+      </c>
+      <c r="B18" t="str">
+        <v>ORD-083726</v>
+      </c>
+      <c r="C18" t="str">
+        <v>17-Jul-2026</v>
+      </c>
+      <c r="D18">
+        <v>40</v>
+      </c>
+      <c r="E18">
+        <v>4</v>
+      </c>
+      <c r="F18">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Kenneth</v>
+      </c>
+      <c r="B19" t="str">
+        <v>ORD-083736</v>
+      </c>
+      <c r="C19" t="str">
+        <v>17-Jul-2026</v>
+      </c>
+      <c r="D19">
+        <v>16</v>
+      </c>
+      <c r="E19">
+        <v>4</v>
+      </c>
+      <c r="F19">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Kenneth</v>
+      </c>
+      <c r="B20" t="str">
+        <v>ORD-084050</v>
+      </c>
+      <c r="C20" t="str">
+        <v>17-Jul-2026</v>
+      </c>
+      <c r="D20">
+        <v>55.5</v>
+      </c>
+      <c r="E20">
+        <v>4</v>
+      </c>
+      <c r="F20">
+        <v>51.5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Kenneth</v>
+      </c>
+      <c r="B21" t="str">
+        <v>ORD-084069</v>
+      </c>
+      <c r="C21" t="str">
+        <v>17-Jul-2026</v>
+      </c>
+      <c r="D21">
+        <v>147</v>
+      </c>
+      <c r="E21">
+        <v>4</v>
+      </c>
+      <c r="F21">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Lawrence Kumah</v>
+      </c>
+      <c r="B22" t="str">
+        <v>ORD-081742</v>
+      </c>
+      <c r="C22" t="str">
+        <v>14-Jul-2026</v>
+      </c>
+      <c r="D22">
+        <v>198.5</v>
+      </c>
+      <c r="E22">
+        <v>190.5</v>
+      </c>
+      <c r="F22">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Notify</v>
+      </c>
+      <c r="B23" t="str">
+        <v>ORD-082326</v>
+      </c>
+      <c r="C23" t="str">
+        <v>15-Jul-2026</v>
+      </c>
+      <c r="D23">
+        <v>43.5</v>
+      </c>
+      <c r="E23">
+        <v>4</v>
+      </c>
+      <c r="F23">
+        <v>39.5</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Notify</v>
+      </c>
+      <c r="B24" t="str">
+        <v>ORD-082485</v>
+      </c>
+      <c r="C24" t="str">
+        <v>15-Jul-2026</v>
+      </c>
+      <c r="D24">
+        <v>16</v>
+      </c>
+      <c r="E24">
+        <v>8</v>
+      </c>
+      <c r="F24">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Notify</v>
+      </c>
+      <c r="B25" t="str">
+        <v>ORD-082909</v>
+      </c>
+      <c r="C25" t="str">
+        <v>16-Jul-2026</v>
+      </c>
+      <c r="D25">
+        <v>55.5</v>
+      </c>
+      <c r="E25">
+        <v>16</v>
+      </c>
+      <c r="F25">
+        <v>39.5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Notify</v>
+      </c>
+      <c r="B26" t="str">
+        <v>ORD-083009</v>
+      </c>
+      <c r="C26" t="str">
+        <v>16-Jul-2026</v>
+      </c>
+      <c r="D26">
+        <v>79.5</v>
+      </c>
+      <c r="E26">
+        <v>8</v>
+      </c>
+      <c r="F26">
+        <v>71.5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Notify</v>
+      </c>
+      <c r="B27" t="str">
+        <v>ORD-083228</v>
+      </c>
+      <c r="C27" t="str">
+        <v>16-Jul-2026</v>
+      </c>
+      <c r="D27">
+        <v>40</v>
+      </c>
+      <c r="E27">
+        <v>20</v>
+      </c>
+      <c r="F27">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Notify</v>
+      </c>
+      <c r="B28" t="str">
+        <v>ORD-083238</v>
+      </c>
+      <c r="C28" t="str">
+        <v>16-Jul-2026</v>
+      </c>
+      <c r="D28">
+        <v>36</v>
+      </c>
+      <c r="E28">
+        <v>4</v>
+      </c>
+      <c r="F28">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Notify</v>
+      </c>
+      <c r="B29" t="str">
+        <v>ORD-083560</v>
+      </c>
+      <c r="C29" t="str">
+        <v>17-Jul-2026</v>
+      </c>
+      <c r="D29">
+        <v>144.5</v>
+      </c>
+      <c r="E29">
+        <v>8</v>
+      </c>
+      <c r="F29">
+        <v>107.45</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F29"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F7"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Agent</v>
       </c>
       <c r="B1" t="str">
         <v>Email</v>
       </c>
       <c r="C1" t="str">
-        <v>Balance Before Deduction (GHS)</v>
+        <v>Balance Before (GHS)</v>
       </c>
       <c r="D1" t="str">
-        <v>Amount Deducted (GHS)</v>
+        <v>Total Recovered (GHS)</v>
       </c>
       <c r="E1" t="str">
         <v>Current Balance (GHS)</v>

</xml_diff>

<commit_message>
Add affected phone number to recovery report
Add recipient phone number column to the over_refund_recovery_20Jul2026.xlsx report by querying the order_items table.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 7cdd434c-ed09-4143-9d63-3c20e2d8d6b0
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 5a48dc1e-711f-4946-bcb5-74dfa1be5e0e
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/348b80b5-3718-405c-9777-744d35985801/7cdd434c-ed09-4143-9d63-3c20e2d8d6b0/hRxk6j6
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/over_refund_recovery_20Jul2026.xlsx
+++ b/over_refund_recovery_20Jul2026.xlsx
@@ -398,14 +398,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:G29"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
     <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="28.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -419,12 +420,15 @@
         <v>Order Placed Date</v>
       </c>
       <c r="D1" t="str">
+        <v>Affected Phone</v>
+      </c>
+      <c r="E1" t="str">
         <v>Amount Refunded (GHS)</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Correct Refund (GHS)</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Over-Refund Recovered (GHS)</v>
       </c>
     </row>
@@ -438,13 +442,16 @@
       <c r="C2" t="str">
         <v>15-Jul-2026</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="str">
+        <v>0539309232</v>
+      </c>
+      <c r="E2">
         <v>12</v>
       </c>
-      <c r="E2">
-        <v>4</v>
-      </c>
       <c r="F2">
+        <v>4</v>
+      </c>
+      <c r="G2">
         <v>3.8</v>
       </c>
     </row>
@@ -458,13 +465,16 @@
       <c r="C3" t="str">
         <v>18-Jul-2026</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="str">
+        <v>0554741943</v>
+      </c>
+      <c r="E3">
         <v>80</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>40</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>1.6</v>
       </c>
     </row>
@@ -478,13 +488,16 @@
       <c r="C4" t="str">
         <v>14-Jul-2026</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="str">
+        <v>0596722230</v>
+      </c>
+      <c r="E4">
         <v>16</v>
       </c>
-      <c r="E4">
-        <v>4</v>
-      </c>
       <c r="F4">
+        <v>4</v>
+      </c>
+      <c r="G4">
         <v>12</v>
       </c>
     </row>
@@ -498,13 +511,16 @@
       <c r="C5" t="str">
         <v>15-Jul-2026</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="str">
+        <v>0596722230</v>
+      </c>
+      <c r="E5">
         <v>8</v>
       </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
       <c r="F5">
+        <v>4</v>
+      </c>
+      <c r="G5">
         <v>4</v>
       </c>
     </row>
@@ -518,13 +534,16 @@
       <c r="C6" t="str">
         <v>15-Jul-2026</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="str">
+        <v>0591728341</v>
+      </c>
+      <c r="E6">
         <v>47.5</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>39.5</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>8</v>
       </c>
     </row>
@@ -538,13 +557,16 @@
       <c r="C7" t="str">
         <v>16-Jul-2026</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="str">
+        <v>0256656521</v>
+      </c>
+      <c r="E7">
         <v>20</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>8</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>12</v>
       </c>
     </row>
@@ -558,13 +580,16 @@
       <c r="C8" t="str">
         <v>16-Jul-2026</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="str">
+        <v>0534512754</v>
+      </c>
+      <c r="E8">
         <v>8</v>
       </c>
-      <c r="E8">
-        <v>4</v>
-      </c>
       <c r="F8">
+        <v>4</v>
+      </c>
+      <c r="G8">
         <v>4</v>
       </c>
     </row>
@@ -578,13 +603,16 @@
       <c r="C9" t="str">
         <v>16-Jul-2026</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="str">
+        <v>0536077442</v>
+      </c>
+      <c r="E9">
         <v>24</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <v>16</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <v>8</v>
       </c>
     </row>
@@ -598,13 +626,16 @@
       <c r="C10" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="str">
+        <v>0548250560</v>
+      </c>
+      <c r="E10">
         <v>44</v>
       </c>
-      <c r="E10">
-        <v>4</v>
-      </c>
       <c r="F10">
+        <v>4</v>
+      </c>
+      <c r="G10">
         <v>40</v>
       </c>
     </row>
@@ -618,13 +649,16 @@
       <c r="C11" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D11">
+      <c r="D11" t="str">
+        <v>0541178542</v>
+      </c>
+      <c r="E11">
         <v>73</v>
       </c>
-      <c r="E11">
-        <v>4</v>
-      </c>
       <c r="F11">
+        <v>4</v>
+      </c>
+      <c r="G11">
         <v>69</v>
       </c>
     </row>
@@ -638,13 +672,16 @@
       <c r="C12" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D12">
+      <c r="D12" t="str">
+        <v>0598435823</v>
+      </c>
+      <c r="E12">
         <v>191</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>20</v>
       </c>
-      <c r="F12">
+      <c r="G12">
         <v>171</v>
       </c>
     </row>
@@ -658,13 +695,16 @@
       <c r="C13" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D13">
+      <c r="D13" t="str">
+        <v>0535506290</v>
+      </c>
+      <c r="E13">
         <v>36</v>
       </c>
-      <c r="E13">
-        <v>4</v>
-      </c>
       <c r="F13">
+        <v>4</v>
+      </c>
+      <c r="G13">
         <v>32</v>
       </c>
     </row>
@@ -678,13 +718,16 @@
       <c r="C14" t="str">
         <v>18-Jul-2026</v>
       </c>
-      <c r="D14">
+      <c r="D14" t="str">
+        <v>0531471459</v>
+      </c>
+      <c r="E14">
         <v>279.5</v>
       </c>
-      <c r="E14">
+      <c r="F14">
         <v>4.1</v>
       </c>
-      <c r="F14">
+      <c r="G14">
         <v>275.4</v>
       </c>
     </row>
@@ -698,13 +741,16 @@
       <c r="C15" t="str">
         <v>18-Jul-2026</v>
       </c>
-      <c r="D15">
+      <c r="D15" t="str">
+        <v>0245260945</v>
+      </c>
+      <c r="E15">
         <v>16.4</v>
       </c>
-      <c r="E15">
+      <c r="F15">
         <v>4.1</v>
       </c>
-      <c r="F15">
+      <c r="G15">
         <v>12.3</v>
       </c>
     </row>
@@ -718,13 +764,16 @@
       <c r="C16" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D16">
+      <c r="D16" t="str">
+        <v>0541996805</v>
+      </c>
+      <c r="E16">
         <v>116</v>
       </c>
-      <c r="E16">
-        <v>4</v>
-      </c>
       <c r="F16">
+        <v>4</v>
+      </c>
+      <c r="G16">
         <v>112</v>
       </c>
     </row>
@@ -738,13 +787,16 @@
       <c r="C17" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D17">
+      <c r="D17" t="str">
+        <v>0556953936</v>
+      </c>
+      <c r="E17">
         <v>24</v>
       </c>
-      <c r="E17">
-        <v>4</v>
-      </c>
       <c r="F17">
+        <v>4</v>
+      </c>
+      <c r="G17">
         <v>20</v>
       </c>
     </row>
@@ -758,13 +810,16 @@
       <c r="C18" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D18">
+      <c r="D18" t="str">
+        <v>0594140707</v>
+      </c>
+      <c r="E18">
         <v>40</v>
       </c>
-      <c r="E18">
-        <v>4</v>
-      </c>
       <c r="F18">
+        <v>4</v>
+      </c>
+      <c r="G18">
         <v>36</v>
       </c>
     </row>
@@ -778,13 +833,16 @@
       <c r="C19" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D19">
+      <c r="D19" t="str">
+        <v>0548014118</v>
+      </c>
+      <c r="E19">
         <v>16</v>
       </c>
-      <c r="E19">
-        <v>4</v>
-      </c>
       <c r="F19">
+        <v>4</v>
+      </c>
+      <c r="G19">
         <v>12</v>
       </c>
     </row>
@@ -798,13 +856,16 @@
       <c r="C20" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D20">
+      <c r="D20" t="str">
+        <v>0555480630</v>
+      </c>
+      <c r="E20">
         <v>55.5</v>
       </c>
-      <c r="E20">
-        <v>4</v>
-      </c>
       <c r="F20">
+        <v>4</v>
+      </c>
+      <c r="G20">
         <v>51.5</v>
       </c>
     </row>
@@ -818,13 +879,16 @@
       <c r="C21" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D21">
+      <c r="D21" t="str">
+        <v>0549536637</v>
+      </c>
+      <c r="E21">
         <v>147</v>
       </c>
-      <c r="E21">
-        <v>4</v>
-      </c>
       <c r="F21">
+        <v>4</v>
+      </c>
+      <c r="G21">
         <v>143</v>
       </c>
     </row>
@@ -838,13 +902,16 @@
       <c r="C22" t="str">
         <v>14-Jul-2026</v>
       </c>
-      <c r="D22">
+      <c r="D22" t="str">
+        <v>0535859740</v>
+      </c>
+      <c r="E22">
         <v>198.5</v>
       </c>
-      <c r="E22">
+      <c r="F22">
         <v>190.5</v>
       </c>
-      <c r="F22">
+      <c r="G22">
         <v>8</v>
       </c>
     </row>
@@ -858,13 +925,16 @@
       <c r="C23" t="str">
         <v>15-Jul-2026</v>
       </c>
-      <c r="D23">
+      <c r="D23" t="str">
+        <v>0531396080</v>
+      </c>
+      <c r="E23">
         <v>43.5</v>
       </c>
-      <c r="E23">
-        <v>4</v>
-      </c>
       <c r="F23">
+        <v>4</v>
+      </c>
+      <c r="G23">
         <v>39.5</v>
       </c>
     </row>
@@ -878,13 +948,16 @@
       <c r="C24" t="str">
         <v>15-Jul-2026</v>
       </c>
-      <c r="D24">
+      <c r="D24" t="str">
+        <v>0596055264</v>
+      </c>
+      <c r="E24">
         <v>16</v>
       </c>
-      <c r="E24">
+      <c r="F24">
         <v>8</v>
       </c>
-      <c r="F24">
+      <c r="G24">
         <v>8</v>
       </c>
     </row>
@@ -898,13 +971,16 @@
       <c r="C25" t="str">
         <v>16-Jul-2026</v>
       </c>
-      <c r="D25">
+      <c r="D25" t="str">
+        <v>0547346638</v>
+      </c>
+      <c r="E25">
         <v>55.5</v>
       </c>
-      <c r="E25">
+      <c r="F25">
         <v>16</v>
       </c>
-      <c r="F25">
+      <c r="G25">
         <v>39.5</v>
       </c>
     </row>
@@ -918,13 +994,16 @@
       <c r="C26" t="str">
         <v>16-Jul-2026</v>
       </c>
-      <c r="D26">
+      <c r="D26" t="str">
+        <v>0243534814</v>
+      </c>
+      <c r="E26">
         <v>79.5</v>
       </c>
-      <c r="E26">
+      <c r="F26">
         <v>8</v>
       </c>
-      <c r="F26">
+      <c r="G26">
         <v>71.5</v>
       </c>
     </row>
@@ -938,13 +1017,16 @@
       <c r="C27" t="str">
         <v>16-Jul-2026</v>
       </c>
-      <c r="D27">
+      <c r="D27" t="str">
+        <v>0553986469</v>
+      </c>
+      <c r="E27">
         <v>40</v>
       </c>
-      <c r="E27">
+      <c r="F27">
         <v>20</v>
       </c>
-      <c r="F27">
+      <c r="G27">
         <v>20</v>
       </c>
     </row>
@@ -958,13 +1040,16 @@
       <c r="C28" t="str">
         <v>16-Jul-2026</v>
       </c>
-      <c r="D28">
+      <c r="D28" t="str">
+        <v>0538659128</v>
+      </c>
+      <c r="E28">
         <v>36</v>
       </c>
-      <c r="E28">
-        <v>4</v>
-      </c>
       <c r="F28">
+        <v>4</v>
+      </c>
+      <c r="G28">
         <v>32</v>
       </c>
     </row>
@@ -978,19 +1063,22 @@
       <c r="C29" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D29">
+      <c r="D29" t="str">
+        <v>0597353350</v>
+      </c>
+      <c r="E29">
         <v>144.5</v>
       </c>
-      <c r="E29">
+      <c r="F29">
         <v>8</v>
       </c>
-      <c r="F29">
+      <c r="G29">
         <v>107.45</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G29"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add bulk admin recovery entries to order breakdown report
Add missing bulk admin recovery entries to the `over_refund_recovery_20Jul2026.xlsx` file, clarifying transaction details for specific agents.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 7cdd434c-ed09-4143-9d63-3c20e2d8d6b0
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: c8be2521-ca72-4646-8e0b-44e53ff10e21
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/348b80b5-3718-405c-9777-744d35985801/7cdd434c-ed09-4143-9d63-3c20e2d8d6b0/hRxk6j6
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/over_refund_recovery_20Jul2026.xlsx
+++ b/over_refund_recovery_20Jul2026.xlsx
@@ -398,15 +398,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:H34"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="28.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -414,21 +415,24 @@
         <v>Agent</v>
       </c>
       <c r="B1" t="str">
+        <v>Type</v>
+      </c>
+      <c r="C1" t="str">
         <v>Order ID</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Order Placed Date</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Affected Phone</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Amount Refunded (GHS)</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Correct Refund (GHS)</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Over-Refund Recovered (GHS)</v>
       </c>
     </row>
@@ -437,21 +441,24 @@
         <v>Dela Kwesi</v>
       </c>
       <c r="B2" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C2" t="str">
         <v>ORD-082506</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>15-Jul-2026</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>0539309232</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>12</v>
       </c>
-      <c r="F2">
-        <v>4</v>
-      </c>
       <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
         <v>3.8</v>
       </c>
     </row>
@@ -460,21 +467,24 @@
         <v>Emmanuel Simpson</v>
       </c>
       <c r="B3" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C3" t="str">
         <v>ORD-084475</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>18-Jul-2026</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>0554741943</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>80</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>40</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>1.6</v>
       </c>
     </row>
@@ -483,21 +493,24 @@
         <v>Flashdealsgh</v>
       </c>
       <c r="B4" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C4" t="str">
         <v>ORD-082068</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>14-Jul-2026</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>0596722230</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>16</v>
       </c>
-      <c r="F4">
-        <v>4</v>
-      </c>
       <c r="G4">
+        <v>4</v>
+      </c>
+      <c r="H4">
         <v>12</v>
       </c>
     </row>
@@ -506,21 +519,24 @@
         <v>Flashdealsgh</v>
       </c>
       <c r="B5" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C5" t="str">
         <v>ORD-082673</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
         <v>15-Jul-2026</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>0596722230</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>8</v>
       </c>
-      <c r="F5">
-        <v>4</v>
-      </c>
       <c r="G5">
+        <v>4</v>
+      </c>
+      <c r="H5">
         <v>4</v>
       </c>
     </row>
@@ -529,21 +545,24 @@
         <v>Flashdealsgh</v>
       </c>
       <c r="B6" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C6" t="str">
         <v>ORD-082739</v>
       </c>
-      <c r="C6" t="str">
+      <c r="D6" t="str">
         <v>15-Jul-2026</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>0591728341</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>47.5</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>39.5</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>8</v>
       </c>
     </row>
@@ -552,21 +571,24 @@
         <v>Flashdealsgh</v>
       </c>
       <c r="B7" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C7" t="str">
         <v>ORD-082838</v>
       </c>
-      <c r="C7" t="str">
+      <c r="D7" t="str">
         <v>16-Jul-2026</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>0256656521</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>20</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>8</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>12</v>
       </c>
     </row>
@@ -575,21 +597,24 @@
         <v>Flashdealsgh</v>
       </c>
       <c r="B8" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C8" t="str">
         <v>ORD-083155</v>
       </c>
-      <c r="C8" t="str">
+      <c r="D8" t="str">
         <v>16-Jul-2026</v>
       </c>
-      <c r="D8" t="str">
+      <c r="E8" t="str">
         <v>0534512754</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>8</v>
       </c>
-      <c r="F8">
-        <v>4</v>
-      </c>
       <c r="G8">
+        <v>4</v>
+      </c>
+      <c r="H8">
         <v>4</v>
       </c>
     </row>
@@ -598,21 +623,24 @@
         <v>Flashdealsgh</v>
       </c>
       <c r="B9" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C9" t="str">
         <v>ORD-083419</v>
       </c>
-      <c r="C9" t="str">
+      <c r="D9" t="str">
         <v>16-Jul-2026</v>
       </c>
-      <c r="D9" t="str">
+      <c r="E9" t="str">
         <v>0536077442</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <v>24</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <v>16</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>8</v>
       </c>
     </row>
@@ -621,21 +649,24 @@
         <v>Flashdealsgh</v>
       </c>
       <c r="B10" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C10" t="str">
         <v>ORD-083485</v>
       </c>
-      <c r="C10" t="str">
+      <c r="D10" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D10" t="str">
+      <c r="E10" t="str">
         <v>0548250560</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <v>44</v>
       </c>
-      <c r="F10">
-        <v>4</v>
-      </c>
       <c r="G10">
+        <v>4</v>
+      </c>
+      <c r="H10">
         <v>40</v>
       </c>
     </row>
@@ -644,21 +675,24 @@
         <v>Flashdealsgh</v>
       </c>
       <c r="B11" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C11" t="str">
         <v>ORD-083539</v>
       </c>
-      <c r="C11" t="str">
+      <c r="D11" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D11" t="str">
+      <c r="E11" t="str">
         <v>0541178542</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <v>73</v>
       </c>
-      <c r="F11">
-        <v>4</v>
-      </c>
       <c r="G11">
+        <v>4</v>
+      </c>
+      <c r="H11">
         <v>69</v>
       </c>
     </row>
@@ -667,21 +701,24 @@
         <v>Flashdealsgh</v>
       </c>
       <c r="B12" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C12" t="str">
         <v>ORD-084002</v>
       </c>
-      <c r="C12" t="str">
+      <c r="D12" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D12" t="str">
+      <c r="E12" t="str">
         <v>0598435823</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>191</v>
       </c>
-      <c r="F12">
+      <c r="G12">
         <v>20</v>
       </c>
-      <c r="G12">
+      <c r="H12">
         <v>171</v>
       </c>
     </row>
@@ -690,21 +727,24 @@
         <v>Flashdealsgh</v>
       </c>
       <c r="B13" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C13" t="str">
         <v>ORD-084042</v>
       </c>
-      <c r="C13" t="str">
+      <c r="D13" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D13" t="str">
+      <c r="E13" t="str">
         <v>0535506290</v>
       </c>
-      <c r="E13">
+      <c r="F13">
         <v>36</v>
       </c>
-      <c r="F13">
-        <v>4</v>
-      </c>
       <c r="G13">
+        <v>4</v>
+      </c>
+      <c r="H13">
         <v>32</v>
       </c>
     </row>
@@ -713,21 +753,24 @@
         <v>Flashdealsgh</v>
       </c>
       <c r="B14" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C14" t="str">
         <v>ORD-084241</v>
       </c>
-      <c r="C14" t="str">
+      <c r="D14" t="str">
         <v>18-Jul-2026</v>
       </c>
-      <c r="D14" t="str">
+      <c r="E14" t="str">
         <v>0531471459</v>
       </c>
-      <c r="E14">
+      <c r="F14">
         <v>279.5</v>
       </c>
-      <c r="F14">
+      <c r="G14">
         <v>4.1</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <v>275.4</v>
       </c>
     </row>
@@ -736,21 +779,24 @@
         <v>Flashdealsgh</v>
       </c>
       <c r="B15" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C15" t="str">
         <v>ORD-084592</v>
       </c>
-      <c r="C15" t="str">
+      <c r="D15" t="str">
         <v>18-Jul-2026</v>
       </c>
-      <c r="D15" t="str">
+      <c r="E15" t="str">
         <v>0245260945</v>
       </c>
-      <c r="E15">
+      <c r="F15">
         <v>16.4</v>
       </c>
-      <c r="F15">
+      <c r="G15">
         <v>4.1</v>
       </c>
-      <c r="G15">
+      <c r="H15">
         <v>12.3</v>
       </c>
     </row>
@@ -759,21 +805,24 @@
         <v>Kenneth</v>
       </c>
       <c r="B16" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C16" t="str">
         <v>ORD-083558</v>
       </c>
-      <c r="C16" t="str">
+      <c r="D16" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D16" t="str">
+      <c r="E16" t="str">
         <v>0541996805</v>
       </c>
-      <c r="E16">
+      <c r="F16">
         <v>116</v>
       </c>
-      <c r="F16">
-        <v>4</v>
-      </c>
       <c r="G16">
+        <v>4</v>
+      </c>
+      <c r="H16">
         <v>112</v>
       </c>
     </row>
@@ -782,21 +831,24 @@
         <v>Kenneth</v>
       </c>
       <c r="B17" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C17" t="str">
         <v>ORD-083636</v>
       </c>
-      <c r="C17" t="str">
+      <c r="D17" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D17" t="str">
+      <c r="E17" t="str">
         <v>0556953936</v>
       </c>
-      <c r="E17">
+      <c r="F17">
         <v>24</v>
       </c>
-      <c r="F17">
-        <v>4</v>
-      </c>
       <c r="G17">
+        <v>4</v>
+      </c>
+      <c r="H17">
         <v>20</v>
       </c>
     </row>
@@ -805,21 +857,24 @@
         <v>Kenneth</v>
       </c>
       <c r="B18" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C18" t="str">
         <v>ORD-083726</v>
       </c>
-      <c r="C18" t="str">
+      <c r="D18" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D18" t="str">
+      <c r="E18" t="str">
         <v>0594140707</v>
       </c>
-      <c r="E18">
+      <c r="F18">
         <v>40</v>
       </c>
-      <c r="F18">
-        <v>4</v>
-      </c>
       <c r="G18">
+        <v>4</v>
+      </c>
+      <c r="H18">
         <v>36</v>
       </c>
     </row>
@@ -828,21 +883,24 @@
         <v>Kenneth</v>
       </c>
       <c r="B19" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C19" t="str">
         <v>ORD-083736</v>
       </c>
-      <c r="C19" t="str">
+      <c r="D19" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D19" t="str">
+      <c r="E19" t="str">
         <v>0548014118</v>
       </c>
-      <c r="E19">
+      <c r="F19">
         <v>16</v>
       </c>
-      <c r="F19">
-        <v>4</v>
-      </c>
       <c r="G19">
+        <v>4</v>
+      </c>
+      <c r="H19">
         <v>12</v>
       </c>
     </row>
@@ -851,21 +909,24 @@
         <v>Kenneth</v>
       </c>
       <c r="B20" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C20" t="str">
         <v>ORD-084050</v>
       </c>
-      <c r="C20" t="str">
+      <c r="D20" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D20" t="str">
+      <c r="E20" t="str">
         <v>0555480630</v>
       </c>
-      <c r="E20">
+      <c r="F20">
         <v>55.5</v>
       </c>
-      <c r="F20">
-        <v>4</v>
-      </c>
       <c r="G20">
+        <v>4</v>
+      </c>
+      <c r="H20">
         <v>51.5</v>
       </c>
     </row>
@@ -874,21 +935,24 @@
         <v>Kenneth</v>
       </c>
       <c r="B21" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C21" t="str">
         <v>ORD-084069</v>
       </c>
-      <c r="C21" t="str">
+      <c r="D21" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D21" t="str">
+      <c r="E21" t="str">
         <v>0549536637</v>
       </c>
-      <c r="E21">
+      <c r="F21">
         <v>147</v>
       </c>
-      <c r="F21">
-        <v>4</v>
-      </c>
       <c r="G21">
+        <v>4</v>
+      </c>
+      <c r="H21">
         <v>143</v>
       </c>
     </row>
@@ -897,21 +961,24 @@
         <v>Lawrence Kumah</v>
       </c>
       <c r="B22" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C22" t="str">
         <v>ORD-081742</v>
       </c>
-      <c r="C22" t="str">
+      <c r="D22" t="str">
         <v>14-Jul-2026</v>
       </c>
-      <c r="D22" t="str">
+      <c r="E22" t="str">
         <v>0535859740</v>
       </c>
-      <c r="E22">
+      <c r="F22">
         <v>198.5</v>
       </c>
-      <c r="F22">
+      <c r="G22">
         <v>190.5</v>
       </c>
-      <c r="G22">
+      <c r="H22">
         <v>8</v>
       </c>
     </row>
@@ -920,21 +987,24 @@
         <v>Notify</v>
       </c>
       <c r="B23" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C23" t="str">
         <v>ORD-082326</v>
       </c>
-      <c r="C23" t="str">
+      <c r="D23" t="str">
         <v>15-Jul-2026</v>
       </c>
-      <c r="D23" t="str">
+      <c r="E23" t="str">
         <v>0531396080</v>
       </c>
-      <c r="E23">
+      <c r="F23">
         <v>43.5</v>
       </c>
-      <c r="F23">
-        <v>4</v>
-      </c>
       <c r="G23">
+        <v>4</v>
+      </c>
+      <c r="H23">
         <v>39.5</v>
       </c>
     </row>
@@ -943,21 +1013,24 @@
         <v>Notify</v>
       </c>
       <c r="B24" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C24" t="str">
         <v>ORD-082485</v>
       </c>
-      <c r="C24" t="str">
+      <c r="D24" t="str">
         <v>15-Jul-2026</v>
       </c>
-      <c r="D24" t="str">
+      <c r="E24" t="str">
         <v>0596055264</v>
       </c>
-      <c r="E24">
+      <c r="F24">
         <v>16</v>
       </c>
-      <c r="F24">
+      <c r="G24">
         <v>8</v>
       </c>
-      <c r="G24">
+      <c r="H24">
         <v>8</v>
       </c>
     </row>
@@ -966,21 +1039,24 @@
         <v>Notify</v>
       </c>
       <c r="B25" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C25" t="str">
         <v>ORD-082909</v>
       </c>
-      <c r="C25" t="str">
+      <c r="D25" t="str">
         <v>16-Jul-2026</v>
       </c>
-      <c r="D25" t="str">
+      <c r="E25" t="str">
         <v>0547346638</v>
       </c>
-      <c r="E25">
+      <c r="F25">
         <v>55.5</v>
       </c>
-      <c r="F25">
+      <c r="G25">
         <v>16</v>
       </c>
-      <c r="G25">
+      <c r="H25">
         <v>39.5</v>
       </c>
     </row>
@@ -989,21 +1065,24 @@
         <v>Notify</v>
       </c>
       <c r="B26" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C26" t="str">
         <v>ORD-083009</v>
       </c>
-      <c r="C26" t="str">
+      <c r="D26" t="str">
         <v>16-Jul-2026</v>
       </c>
-      <c r="D26" t="str">
+      <c r="E26" t="str">
         <v>0243534814</v>
       </c>
-      <c r="E26">
+      <c r="F26">
         <v>79.5</v>
       </c>
-      <c r="F26">
+      <c r="G26">
         <v>8</v>
       </c>
-      <c r="G26">
+      <c r="H26">
         <v>71.5</v>
       </c>
     </row>
@@ -1012,21 +1091,24 @@
         <v>Notify</v>
       </c>
       <c r="B27" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C27" t="str">
         <v>ORD-083228</v>
       </c>
-      <c r="C27" t="str">
+      <c r="D27" t="str">
         <v>16-Jul-2026</v>
       </c>
-      <c r="D27" t="str">
+      <c r="E27" t="str">
         <v>0553986469</v>
       </c>
-      <c r="E27">
+      <c r="F27">
         <v>40</v>
       </c>
-      <c r="F27">
+      <c r="G27">
         <v>20</v>
       </c>
-      <c r="G27">
+      <c r="H27">
         <v>20</v>
       </c>
     </row>
@@ -1035,21 +1117,24 @@
         <v>Notify</v>
       </c>
       <c r="B28" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C28" t="str">
         <v>ORD-083238</v>
       </c>
-      <c r="C28" t="str">
+      <c r="D28" t="str">
         <v>16-Jul-2026</v>
       </c>
-      <c r="D28" t="str">
+      <c r="E28" t="str">
         <v>0538659128</v>
       </c>
-      <c r="E28">
+      <c r="F28">
         <v>36</v>
       </c>
-      <c r="F28">
-        <v>4</v>
-      </c>
       <c r="G28">
+        <v>4</v>
+      </c>
+      <c r="H28">
         <v>32</v>
       </c>
     </row>
@@ -1058,27 +1143,160 @@
         <v>Notify</v>
       </c>
       <c r="B29" t="str">
+        <v>Order Recovery</v>
+      </c>
+      <c r="C29" t="str">
         <v>ORD-083560</v>
       </c>
-      <c r="C29" t="str">
+      <c r="D29" t="str">
         <v>17-Jul-2026</v>
       </c>
-      <c r="D29" t="str">
+      <c r="E29" t="str">
         <v>0597353350</v>
       </c>
-      <c r="E29">
+      <c r="F29">
         <v>144.5</v>
       </c>
-      <c r="F29">
+      <c r="G29">
         <v>8</v>
       </c>
-      <c r="G29">
+      <c r="H29">
         <v>107.45</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Flashdealsgh</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Bulk Admin Correction</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Bulk Admin Correction</v>
+      </c>
+      <c r="D30" t="str">
+        <v>20-Jul-2026</v>
+      </c>
+      <c r="E30" t="str">
+        <v>—</v>
+      </c>
+      <c r="F30" t="str">
+        <v>—</v>
+      </c>
+      <c r="G30" t="str">
+        <v>—</v>
+      </c>
+      <c r="H30">
+        <v>607.6</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Kenneth</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Bulk Admin Correction</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Bulk Admin Correction</v>
+      </c>
+      <c r="D31" t="str">
+        <v>20-Jul-2026</v>
+      </c>
+      <c r="E31" t="str">
+        <v>—</v>
+      </c>
+      <c r="F31" t="str">
+        <v>—</v>
+      </c>
+      <c r="G31" t="str">
+        <v>—</v>
+      </c>
+      <c r="H31">
+        <v>350.5</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Lawrence Kumah</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Bulk Admin Correction</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Bulk Admin Correction</v>
+      </c>
+      <c r="D32" t="str">
+        <v>20-Jul-2026</v>
+      </c>
+      <c r="E32" t="str">
+        <v>—</v>
+      </c>
+      <c r="F32" t="str">
+        <v>—</v>
+      </c>
+      <c r="G32" t="str">
+        <v>—</v>
+      </c>
+      <c r="H32">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Notify</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Bulk Admin Correction</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Bulk Admin Correction</v>
+      </c>
+      <c r="D33" t="str">
+        <v>20-Jul-2026</v>
+      </c>
+      <c r="E33" t="str">
+        <v>—</v>
+      </c>
+      <c r="F33" t="str">
+        <v>—</v>
+      </c>
+      <c r="G33" t="str">
+        <v>—</v>
+      </c>
+      <c r="H33">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Notify</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Debt Recovery</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Debt Auto-Recovery</v>
+      </c>
+      <c r="D34" t="str">
+        <v>20-Jul-2026</v>
+      </c>
+      <c r="E34" t="str">
+        <v>—</v>
+      </c>
+      <c r="F34" t="str">
+        <v>—</v>
+      </c>
+      <c r="G34" t="str">
+        <v>—</v>
+      </c>
+      <c r="H34">
+        <v>29.05</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H34"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>